<commit_message>
feat: release Checkee data 20260914-v001
</commit_message>
<xml_diff>
--- a/data/checkmate/hall_fame.xlsx
+++ b/data/checkmate/hall_fame.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\projects_2027\checkee_2026\data\checkmate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{847635D8-6011-421A-B7DD-8B262319D0CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F58A4127-BC96-40B9-AAE6-DB08711EB5C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6980" yWindow="5440" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="842" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="282">
   <si>
     <t>地点</t>
   </si>
@@ -156,9 +156,6 @@
   </si>
   <si>
     <t>ufun-checkee-011</t>
-  </si>
-  <si>
-    <t>5.19 update日期，依然lr，initial opt, 还没入职</t>
   </si>
   <si>
     <t>ufun-checkee-012</t>
@@ -214,9 +211,6 @@
   </si>
   <si>
     <t>Emory</t>
-  </si>
-  <si>
-    <t>ufun-checkee-018</t>
   </si>
   <si>
     <t>Columbia</t>
@@ -1747,7 +1741,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S193"/>
+  <dimension ref="A1:S192"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.83203125" style="37" customWidth="1"/>
@@ -1763,7 +1757,7 @@
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A1" s="41" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1796,7 +1790,7 @@
         <v>8</v>
       </c>
       <c r="L1" s="43" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="M1" s="6"/>
       <c r="N1" s="6"/>
@@ -1810,7 +1804,7 @@
     </row>
     <row r="2" spans="1:19" s="37" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="45" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>10</v>
@@ -1847,7 +1841,7 @@
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A3" s="41" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>10</v>
@@ -1856,7 +1850,7 @@
         <v>16</v>
       </c>
       <c r="D3" s="34" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="E3" s="38" t="s">
         <v>13</v>
@@ -1869,10 +1863,10 @@
       </c>
       <c r="H3" s="12"/>
       <c r="I3" s="34" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="J3" s="34" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="K3" s="6"/>
       <c r="L3" s="6"/>
@@ -1888,7 +1882,7 @@
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A4" s="45" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>10</v>
@@ -1927,7 +1921,7 @@
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A5" s="45" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>10</v>
@@ -1936,7 +1930,7 @@
         <v>16</v>
       </c>
       <c r="D5" s="34" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>17</v>
@@ -1949,10 +1943,10 @@
       </c>
       <c r="H5" s="13"/>
       <c r="I5" s="34" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="J5" s="34" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="K5" s="6"/>
       <c r="L5" s="6"/>
@@ -1968,7 +1962,7 @@
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A6" s="41" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>20</v>
@@ -2005,7 +1999,7 @@
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A7" s="41" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>10</v>
@@ -2014,7 +2008,7 @@
         <v>16</v>
       </c>
       <c r="D7" s="34" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>17</v>
@@ -2027,7 +2021,7 @@
       </c>
       <c r="H7" s="12"/>
       <c r="I7" s="34" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="J7" s="6"/>
       <c r="K7" s="6"/>
@@ -2044,7 +2038,7 @@
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A8" s="41" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>10</v>
@@ -2085,7 +2079,7 @@
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A9" s="41" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>10</v>
@@ -2107,7 +2101,7 @@
       </c>
       <c r="H9" s="12"/>
       <c r="I9" s="34" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="J9" s="6"/>
       <c r="K9" s="6"/>
@@ -2164,7 +2158,7 @@
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A11" s="45" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>10</v>
@@ -2173,7 +2167,7 @@
         <v>11</v>
       </c>
       <c r="D11" s="34" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E11" s="42" t="s">
         <v>28</v>
@@ -2186,7 +2180,7 @@
       </c>
       <c r="H11" s="12"/>
       <c r="I11" s="34" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="J11" s="6"/>
       <c r="K11" s="6"/>
@@ -2266,7 +2260,7 @@
       <c r="Q13" s="6"/>
       <c r="R13" s="6"/>
       <c r="S13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.35">
@@ -2300,7 +2294,7 @@
       <c r="Q14" s="6"/>
       <c r="R14" s="6"/>
       <c r="S14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.35">
@@ -2338,12 +2332,12 @@
       <c r="Q15" s="6"/>
       <c r="R15" s="6"/>
       <c r="S15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A16" s="41" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>20</v>
@@ -2352,7 +2346,7 @@
         <v>11</v>
       </c>
       <c r="D16" s="34" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>28</v>
@@ -2365,7 +2359,7 @@
       </c>
       <c r="H16" s="12"/>
       <c r="I16" s="34" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="J16" s="34"/>
       <c r="K16" s="6"/>
@@ -2377,7 +2371,7 @@
       <c r="Q16" s="6"/>
       <c r="R16" s="6"/>
       <c r="S16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:19" ht="26" customHeight="1" x14ac:dyDescent="0.35">
@@ -2388,10 +2382,10 @@
         <v>11</v>
       </c>
       <c r="D17" s="34" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F17" s="8">
         <v>46154</v>
@@ -2401,10 +2395,10 @@
       </c>
       <c r="H17" s="12"/>
       <c r="I17" s="34" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="J17" s="34" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="K17" s="6"/>
       <c r="L17" s="6"/>
@@ -2415,7 +2409,7 @@
       <c r="Q17" s="6"/>
       <c r="R17" s="6"/>
       <c r="S17" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.35">
@@ -2451,36 +2445,36 @@
       <c r="Q18" s="6"/>
       <c r="R18" s="6"/>
       <c r="S18" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B19" s="6" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="E19" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F19" s="8">
-        <v>46157</v>
+      <c r="F19" s="11">
+        <v>46161</v>
       </c>
       <c r="G19" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H19" s="12"/>
       <c r="I19" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="J19" s="6"/>
-      <c r="K19" s="6" t="s">
-        <v>41</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="K19" s="6"/>
       <c r="L19" s="6"/>
       <c r="M19" s="6"/>
       <c r="N19" s="6"/>
@@ -2493,6 +2487,9 @@
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A20" s="45" t="s">
+        <v>222</v>
+      </c>
       <c r="B20" s="6" t="s">
         <v>10</v>
       </c>
@@ -2500,7 +2497,7 @@
         <v>16</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E20" s="7" t="s">
         <v>28</v>
@@ -2512,11 +2509,11 @@
         <v>14</v>
       </c>
       <c r="H20" s="12"/>
-      <c r="I20" s="6" t="s">
-        <v>44</v>
+      <c r="I20" s="34" t="s">
+        <v>221</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K20" s="6"/>
       <c r="L20" s="6"/>
@@ -2527,37 +2524,37 @@
       <c r="Q20" s="6"/>
       <c r="R20" s="6"/>
       <c r="S20" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A21" s="45" t="s">
-        <v>224</v>
+        <v>245</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>43</v>
+        <v>11</v>
+      </c>
+      <c r="D21" s="34" t="s">
+        <v>246</v>
       </c>
       <c r="E21" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F21" s="11">
+      <c r="F21" s="8">
         <v>46161</v>
       </c>
       <c r="G21" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H21" s="12"/>
+      <c r="H21" s="13"/>
       <c r="I21" s="34" t="s">
-        <v>223</v>
-      </c>
-      <c r="J21" s="6" t="s">
-        <v>43</v>
+        <v>247</v>
+      </c>
+      <c r="J21" s="34" t="s">
+        <v>246</v>
       </c>
       <c r="K21" s="6"/>
       <c r="L21" s="6"/>
@@ -2568,39 +2565,36 @@
       <c r="Q21" s="6"/>
       <c r="R21" s="6"/>
       <c r="S21" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A22" s="45" t="s">
-        <v>247</v>
-      </c>
       <c r="B22" s="6" t="s">
         <v>20</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D22" s="34" t="s">
-        <v>248</v>
+        <v>16</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="E22" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F22" s="8">
-        <v>46161</v>
+      <c r="F22" s="11">
+        <v>46163</v>
       </c>
       <c r="G22" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H22" s="13"/>
-      <c r="I22" s="34" t="s">
-        <v>249</v>
-      </c>
-      <c r="J22" s="34" t="s">
-        <v>248</v>
-      </c>
-      <c r="K22" s="6"/>
+      <c r="I22" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="J22" s="6"/>
+      <c r="K22" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="L22" s="6"/>
       <c r="M22" s="6"/>
       <c r="N22" s="6"/>
@@ -2609,35 +2603,38 @@
       <c r="Q22" s="6"/>
       <c r="R22" s="6"/>
       <c r="S22" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A23" s="41" t="s">
+        <v>236</v>
+      </c>
       <c r="B23" s="6" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>21</v>
+        <v>11</v>
+      </c>
+      <c r="D23" s="34" t="s">
+        <v>215</v>
       </c>
       <c r="E23" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F23" s="11">
+      <c r="F23" s="8">
         <v>46163</v>
       </c>
       <c r="G23" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H23" s="13"/>
-      <c r="I23" s="6" t="s">
-        <v>46</v>
+      <c r="H23" s="12"/>
+      <c r="I23" s="34" t="s">
+        <v>235</v>
       </c>
       <c r="J23" s="6"/>
-      <c r="K23" s="6" t="s">
-        <v>30</v>
+      <c r="K23" s="34" t="s">
+        <v>237</v>
       </c>
       <c r="L23" s="6"/>
       <c r="M23" s="6"/>
@@ -2651,34 +2648,33 @@
       </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A24" s="41" t="s">
-        <v>238</v>
-      </c>
       <c r="B24" s="6" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D24" s="34" t="s">
-        <v>217</v>
+        <v>16</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>47</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>28</v>
       </c>
       <c r="F24" s="8">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="G24" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H24" s="12"/>
-      <c r="I24" s="34" t="s">
-        <v>237</v>
-      </c>
-      <c r="J24" s="6"/>
-      <c r="K24" s="34" t="s">
-        <v>239</v>
+      <c r="I24" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="J24" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>49</v>
       </c>
       <c r="L24" s="6"/>
       <c r="M24" s="6"/>
@@ -2688,10 +2684,10 @@
       <c r="Q24" s="6"/>
       <c r="R24" s="6"/>
       <c r="S24" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" ht="26" x14ac:dyDescent="0.35">
       <c r="B25" s="6" t="s">
         <v>20</v>
       </c>
@@ -2699,26 +2695,26 @@
         <v>16</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="E25" s="7" t="s">
         <v>28</v>
       </c>
       <c r="F25" s="8">
-        <v>46164</v>
+        <v>46168</v>
       </c>
       <c r="G25" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H25" s="12"/>
+      <c r="H25" s="13"/>
       <c r="I25" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="K25" s="6" t="s">
-        <v>50</v>
+        <v>37</v>
+      </c>
+      <c r="K25" s="14" t="s">
+        <v>52</v>
       </c>
       <c r="L25" s="6"/>
       <c r="M25" s="6"/>
@@ -2728,37 +2724,33 @@
       <c r="Q25" s="6"/>
       <c r="R25" s="6"/>
       <c r="S25" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="26" spans="1:19" ht="26" x14ac:dyDescent="0.35">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B26" s="6" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C26" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D26" s="7" t="s">
-        <v>37</v>
-      </c>
+      <c r="D26" s="7"/>
       <c r="E26" s="7" t="s">
         <v>28</v>
       </c>
       <c r="F26" s="8">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="G26" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H26" s="13"/>
       <c r="I26" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="J26" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="K26" s="14" t="s">
-        <v>53</v>
+        <v>54</v>
+      </c>
+      <c r="J26" s="6"/>
+      <c r="K26" s="6" t="s">
+        <v>55</v>
       </c>
       <c r="L26" s="6"/>
       <c r="M26" s="6"/>
@@ -2768,12 +2760,12 @@
       <c r="Q26" s="6"/>
       <c r="R26" s="6"/>
       <c r="S26" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B27" s="6" t="s">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="C27" s="6" t="s">
         <v>16</v>
@@ -2788,14 +2780,12 @@
       <c r="G27" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H27" s="13"/>
+      <c r="H27" s="12"/>
       <c r="I27" s="6" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J27" s="6"/>
-      <c r="K27" s="6" t="s">
-        <v>56</v>
-      </c>
+      <c r="K27" s="6"/>
       <c r="L27" s="6"/>
       <c r="M27" s="6"/>
       <c r="N27" s="6"/>
@@ -2804,22 +2794,24 @@
       <c r="Q27" s="6"/>
       <c r="R27" s="6"/>
       <c r="S27" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B28" s="6" t="s">
-        <v>58</v>
+        <v>10</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D28" s="7"/>
+        <v>11</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>12</v>
+      </c>
       <c r="E28" s="7" t="s">
         <v>28</v>
       </c>
       <c r="F28" s="8">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="G28" s="7" t="s">
         <v>14</v>
@@ -2843,13 +2835,13 @@
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B29" s="6" t="s">
-        <v>10</v>
+        <v>61</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="E29" s="7" t="s">
         <v>28</v>
@@ -2861,11 +2853,11 @@
         <v>14</v>
       </c>
       <c r="H29" s="12"/>
-      <c r="I29" s="6" t="s">
-        <v>61</v>
-      </c>
+      <c r="I29" s="6"/>
       <c r="J29" s="6"/>
-      <c r="K29" s="6"/>
+      <c r="K29" s="6" t="s">
+        <v>62</v>
+      </c>
       <c r="L29" s="6"/>
       <c r="M29" s="6"/>
       <c r="N29" s="6"/>
@@ -2874,18 +2866,18 @@
       <c r="Q29" s="6"/>
       <c r="R29" s="6"/>
       <c r="S29" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B30" s="6" t="s">
-        <v>63</v>
+        <v>20</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E30" s="7" t="s">
         <v>28</v>
@@ -2897,11 +2889,13 @@
         <v>14</v>
       </c>
       <c r="H30" s="12"/>
-      <c r="I30" s="6"/>
-      <c r="J30" s="6"/>
-      <c r="K30" s="6" t="s">
-        <v>64</v>
-      </c>
+      <c r="I30" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="J30" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="K30" s="6"/>
       <c r="L30" s="6"/>
       <c r="M30" s="6"/>
       <c r="N30" s="6"/>
@@ -2910,35 +2904,31 @@
       <c r="Q30" s="6"/>
       <c r="R30" s="6"/>
       <c r="S30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B31" s="6" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D31" s="7" t="s">
-        <v>37</v>
-      </c>
+      <c r="D31" s="7"/>
       <c r="E31" s="7" t="s">
-        <v>28</v>
+        <v>65</v>
       </c>
       <c r="F31" s="8">
-        <v>46170</v>
+        <v>46174</v>
       </c>
       <c r="G31" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="H31" s="12"/>
-      <c r="I31" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="J31" s="6" t="s">
-        <v>37</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="H31" s="12">
+        <v>46262</v>
+      </c>
+      <c r="I31" s="6"/>
+      <c r="J31" s="6"/>
       <c r="K31" s="6"/>
       <c r="L31" s="6"/>
       <c r="M31" s="6"/>
@@ -2953,25 +2943,27 @@
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B32" s="6" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C32" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D32" s="7"/>
+      <c r="D32" s="7" t="s">
+        <v>35</v>
+      </c>
       <c r="E32" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F32" s="8">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="G32" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H32" s="12"/>
+      <c r="I32" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="H32" s="12">
-        <v>46262</v>
-      </c>
-      <c r="I32" s="6"/>
       <c r="J32" s="6"/>
       <c r="K32" s="6"/>
       <c r="L32" s="6"/>
@@ -2987,16 +2979,16 @@
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B33" s="6" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F33" s="8">
         <v>46175</v>
@@ -3004,10 +2996,8 @@
       <c r="G33" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H33" s="12"/>
-      <c r="I33" s="6" t="s">
-        <v>70</v>
-      </c>
+      <c r="H33" s="13"/>
+      <c r="I33" s="6"/>
       <c r="J33" s="6"/>
       <c r="K33" s="6"/>
       <c r="L33" s="6"/>
@@ -3022,17 +3012,20 @@
       </c>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A34" s="45" t="s">
+        <v>281</v>
+      </c>
       <c r="B34" s="6" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>12</v>
+        <v>71</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F34" s="8">
         <v>46175</v>
@@ -3041,7 +3034,9 @@
         <v>14</v>
       </c>
       <c r="H34" s="13"/>
-      <c r="I34" s="6"/>
+      <c r="I34" s="6" t="s">
+        <v>72</v>
+      </c>
       <c r="J34" s="6"/>
       <c r="K34" s="6"/>
       <c r="L34" s="6"/>
@@ -3052,37 +3047,36 @@
       <c r="Q34" s="6"/>
       <c r="R34" s="6"/>
       <c r="S34" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A35" s="45" t="s">
-        <v>283</v>
-      </c>
       <c r="B35" s="6" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>73</v>
+        <v>12</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F35" s="8">
-        <v>46175</v>
+        <v>46176</v>
       </c>
       <c r="G35" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H35" s="13"/>
-      <c r="I35" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="J35" s="6"/>
-      <c r="K35" s="6"/>
+      <c r="H35" s="12"/>
+      <c r="I35" s="6"/>
+      <c r="J35" s="34" t="s">
+        <v>278</v>
+      </c>
+      <c r="K35" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="L35" s="6"/>
       <c r="M35" s="6"/>
       <c r="N35" s="6"/>
@@ -3091,36 +3085,34 @@
       <c r="Q35" s="6"/>
       <c r="R35" s="6"/>
       <c r="S35" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B36" s="6" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F36" s="8">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="G36" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H36" s="12"/>
-      <c r="I36" s="6"/>
-      <c r="J36" s="34" t="s">
-        <v>280</v>
-      </c>
-      <c r="K36" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="I36" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="J36" s="6"/>
+      <c r="K36" s="6"/>
       <c r="L36" s="6"/>
       <c r="M36" s="6"/>
       <c r="N36" s="6"/>
@@ -3129,86 +3121,86 @@
       <c r="Q36" s="6"/>
       <c r="R36" s="6"/>
       <c r="S36" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="B37" s="6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="37" spans="1:19" s="37" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="41" t="s">
+        <v>275</v>
+      </c>
+      <c r="B37" s="48" t="s">
         <v>20</v>
       </c>
-      <c r="C37" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D37" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="E37" s="7" t="s">
-        <v>67</v>
+      <c r="C37" s="48" t="s">
+        <v>16</v>
+      </c>
+      <c r="D37" s="34" t="s">
+        <v>278</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>65</v>
       </c>
       <c r="F37" s="8">
-        <v>46177</v>
-      </c>
-      <c r="G37" s="7" t="s">
+        <v>46181</v>
+      </c>
+      <c r="G37" s="9" t="s">
         <v>14</v>
       </c>
       <c r="H37" s="12"/>
-      <c r="I37" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="J37" s="6"/>
-      <c r="K37" s="6"/>
-      <c r="L37" s="6"/>
-      <c r="M37" s="6"/>
-      <c r="N37" s="6"/>
-      <c r="O37" s="6"/>
-      <c r="P37" s="6"/>
-      <c r="Q37" s="6"/>
-      <c r="R37" s="6"/>
+      <c r="I37" s="54" t="s">
+        <v>235</v>
+      </c>
+      <c r="J37" s="54" t="s">
+        <v>276</v>
+      </c>
+      <c r="K37" s="54" t="s">
+        <v>277</v>
+      </c>
+      <c r="L37" s="48"/>
+      <c r="M37" s="48"/>
+      <c r="N37" s="48"/>
+      <c r="O37" s="48"/>
+      <c r="P37" s="48"/>
+      <c r="Q37" s="48"/>
+      <c r="R37" s="48"/>
       <c r="S37" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="38" spans="1:19" s="37" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="41" t="s">
-        <v>277</v>
-      </c>
-      <c r="B38" s="48" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="38" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="B38" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C38" s="48" t="s">
+      <c r="C38" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D38" s="34" t="s">
-        <v>280</v>
-      </c>
-      <c r="E38" s="9" t="s">
-        <v>67</v>
+        <v>215</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>65</v>
       </c>
       <c r="F38" s="8">
         <v>46181</v>
       </c>
-      <c r="G38" s="9" t="s">
+      <c r="G38" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H38" s="12"/>
-      <c r="I38" s="54" t="s">
-        <v>237</v>
-      </c>
-      <c r="J38" s="54" t="s">
-        <v>278</v>
-      </c>
-      <c r="K38" s="54" t="s">
-        <v>279</v>
-      </c>
-      <c r="L38" s="48"/>
-      <c r="M38" s="48"/>
-      <c r="N38" s="48"/>
-      <c r="O38" s="48"/>
-      <c r="P38" s="48"/>
-      <c r="Q38" s="48"/>
-      <c r="R38" s="48"/>
+      <c r="I38" s="6"/>
+      <c r="J38" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="K38" s="6"/>
+      <c r="L38" s="6"/>
+      <c r="M38" s="6"/>
+      <c r="N38" s="6"/>
+      <c r="O38" s="6"/>
+      <c r="P38" s="6"/>
+      <c r="Q38" s="6"/>
+      <c r="R38" s="6"/>
       <c r="S38" t="s">
-        <v>281</v>
+        <v>96</v>
       </c>
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.35">
@@ -3216,25 +3208,23 @@
         <v>20</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D39" s="34" t="s">
-        <v>217</v>
+        <v>11</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="F39" s="8">
-        <v>46181</v>
+        <v>65</v>
+      </c>
+      <c r="F39" s="11">
+        <v>46182</v>
       </c>
       <c r="G39" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H39" s="12"/>
       <c r="I39" s="6"/>
-      <c r="J39" s="6" t="s">
-        <v>78</v>
-      </c>
+      <c r="J39" s="6"/>
       <c r="K39" s="6"/>
       <c r="L39" s="6"/>
       <c r="M39" s="6"/>
@@ -3244,7 +3234,7 @@
       <c r="Q39" s="6"/>
       <c r="R39" s="6"/>
       <c r="S39" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="40" spans="1:19" x14ac:dyDescent="0.35">
@@ -3255,12 +3245,12 @@
         <v>11</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="F40" s="11">
+        <v>65</v>
+      </c>
+      <c r="F40" s="8">
         <v>46182</v>
       </c>
       <c r="G40" s="7" t="s">
@@ -3289,10 +3279,10 @@
         <v>11</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>12</v>
+        <v>80</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F41" s="8">
         <v>46182</v>
@@ -3300,9 +3290,13 @@
       <c r="G41" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H41" s="12"/>
-      <c r="I41" s="6"/>
-      <c r="J41" s="6"/>
+      <c r="H41" s="13"/>
+      <c r="I41" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="J41" s="6" t="s">
+        <v>80</v>
+      </c>
       <c r="K41" s="6"/>
       <c r="L41" s="6"/>
       <c r="M41" s="6"/>
@@ -3312,7 +3306,7 @@
       <c r="Q41" s="6"/>
       <c r="R41" s="6"/>
       <c r="S41" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.35">
@@ -3320,13 +3314,13 @@
         <v>20</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D42" s="7" t="s">
         <v>82</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F42" s="8">
         <v>46182</v>
@@ -3335,9 +3329,7 @@
         <v>14</v>
       </c>
       <c r="H42" s="13"/>
-      <c r="I42" s="6" t="s">
-        <v>52</v>
-      </c>
+      <c r="I42" s="6"/>
       <c r="J42" s="6" t="s">
         <v>82</v>
       </c>
@@ -3350,7 +3342,7 @@
       <c r="Q42" s="6"/>
       <c r="R42" s="6"/>
       <c r="S42" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.35">
@@ -3360,11 +3352,9 @@
       <c r="C43" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D43" s="7" t="s">
-        <v>84</v>
-      </c>
+      <c r="D43" s="7"/>
       <c r="E43" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F43" s="8">
         <v>46182</v>
@@ -3372,12 +3362,14 @@
       <c r="G43" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H43" s="13"/>
-      <c r="I43" s="6"/>
-      <c r="J43" s="6" t="s">
+      <c r="H43" s="12"/>
+      <c r="I43" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="K43" s="6"/>
+      <c r="J43" s="6"/>
+      <c r="K43" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="L43" s="6"/>
       <c r="M43" s="6"/>
       <c r="N43" s="6"/>
@@ -3386,7 +3378,7 @@
       <c r="Q43" s="6"/>
       <c r="R43" s="6"/>
       <c r="S43" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.35">
@@ -3394,25 +3386,31 @@
         <v>20</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D44" s="7"/>
+        <v>11</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>86</v>
+      </c>
       <c r="E44" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F44" s="8">
-        <v>46182</v>
+        <v>46183</v>
       </c>
       <c r="G44" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="H44" s="12"/>
-      <c r="I44" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="J44" s="6"/>
-      <c r="K44" s="6" t="s">
-        <v>30</v>
+        <v>87</v>
+      </c>
+      <c r="H44" s="12">
+        <v>46268</v>
+      </c>
+      <c r="I44" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="J44" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="K44" s="34" t="s">
+        <v>90</v>
       </c>
       <c r="L44" s="6"/>
       <c r="M44" s="6"/>
@@ -3422,40 +3420,32 @@
       <c r="Q44" s="6"/>
       <c r="R44" s="6"/>
       <c r="S44" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B45" s="6" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>88</v>
+        <v>12</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F45" s="8">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="G45" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="H45" s="12">
-        <v>46268</v>
-      </c>
-      <c r="I45" s="21" t="s">
-        <v>90</v>
-      </c>
-      <c r="J45" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="K45" s="34" t="s">
-        <v>92</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="H45" s="12"/>
+      <c r="I45" s="6"/>
+      <c r="J45" s="6"/>
+      <c r="K45" s="6"/>
       <c r="L45" s="6"/>
       <c r="M45" s="6"/>
       <c r="N45" s="6"/>
@@ -3464,21 +3454,24 @@
       <c r="Q45" s="6"/>
       <c r="R45" s="6"/>
       <c r="S45" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A46" s="45" t="s">
+        <v>223</v>
+      </c>
       <c r="B46" s="6" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C46" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D46" s="7" t="s">
-        <v>12</v>
+      <c r="D46" s="34" t="s">
+        <v>224</v>
       </c>
       <c r="E46" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F46" s="8">
         <v>46184</v>
@@ -3487,8 +3480,12 @@
         <v>14</v>
       </c>
       <c r="H46" s="12"/>
-      <c r="I46" s="6"/>
-      <c r="J46" s="6"/>
+      <c r="I46" s="34" t="s">
+        <v>225</v>
+      </c>
+      <c r="J46" s="34" t="s">
+        <v>224</v>
+      </c>
       <c r="K46" s="6"/>
       <c r="L46" s="6"/>
       <c r="M46" s="6"/>
@@ -3498,24 +3495,24 @@
       <c r="Q46" s="6"/>
       <c r="R46" s="6"/>
       <c r="S46" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A47" s="45" t="s">
-        <v>225</v>
+      <c r="A47" s="41" t="s">
+        <v>238</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C47" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D47" s="34" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="E47" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F47" s="8">
         <v>46184</v>
@@ -3525,10 +3522,10 @@
       </c>
       <c r="H47" s="12"/>
       <c r="I47" s="34" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
       <c r="J47" s="34" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="K47" s="6"/>
       <c r="L47" s="6"/>
@@ -3539,38 +3536,31 @@
       <c r="Q47" s="6"/>
       <c r="R47" s="6"/>
       <c r="S47" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="48" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A48" s="41" t="s">
-        <v>240</v>
-      </c>
       <c r="B48" s="6" t="s">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D48" s="34" t="s">
-        <v>242</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="D48" s="7"/>
       <c r="E48" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F48" s="8">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="G48" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H48" s="12"/>
-      <c r="I48" s="34" t="s">
-        <v>241</v>
-      </c>
-      <c r="J48" s="34" t="s">
-        <v>242</v>
-      </c>
+      <c r="I48" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="J48" s="6"/>
       <c r="K48" s="6"/>
       <c r="L48" s="6"/>
       <c r="M48" s="6"/>
@@ -3585,27 +3575,33 @@
     </row>
     <row r="49" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B49" s="6" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D49" s="7"/>
+        <v>16</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>94</v>
+      </c>
       <c r="E49" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F49" s="8">
         <v>46185</v>
       </c>
       <c r="G49" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="H49" s="12"/>
-      <c r="I49" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="J49" s="6"/>
-      <c r="K49" s="6"/>
+        <v>66</v>
+      </c>
+      <c r="H49" s="12">
+        <v>46266</v>
+      </c>
+      <c r="I49" s="6"/>
+      <c r="J49" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="K49" s="6" t="s">
+        <v>95</v>
+      </c>
       <c r="L49" s="6"/>
       <c r="M49" s="6"/>
       <c r="N49" s="6"/>
@@ -3619,32 +3615,32 @@
     </row>
     <row r="50" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B50" s="6" t="s">
-        <v>20</v>
+        <v>97</v>
       </c>
       <c r="C50" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D50" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E50" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F50" s="8">
         <v>46185</v>
       </c>
       <c r="G50" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="H50" s="12">
-        <v>46266</v>
-      </c>
-      <c r="I50" s="6"/>
+        <v>14</v>
+      </c>
+      <c r="H50" s="12"/>
+      <c r="I50" s="6" t="s">
+        <v>99</v>
+      </c>
       <c r="J50" s="6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="K50" s="6" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="L50" s="6"/>
       <c r="M50" s="6"/>
@@ -3659,16 +3655,16 @@
     </row>
     <row r="51" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B51" s="6" t="s">
-        <v>99</v>
+        <v>20</v>
       </c>
       <c r="C51" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D51" s="7" t="s">
-        <v>100</v>
+        <v>12</v>
       </c>
       <c r="E51" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F51" s="8">
         <v>46185</v>
@@ -3678,14 +3674,10 @@
       </c>
       <c r="H51" s="12"/>
       <c r="I51" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="J51" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="K51" s="6" t="s">
         <v>102</v>
       </c>
+      <c r="J51" s="6"/>
+      <c r="K51" s="6"/>
       <c r="L51" s="6"/>
       <c r="M51" s="6"/>
       <c r="N51" s="6"/>
@@ -3694,7 +3686,7 @@
       <c r="Q51" s="6"/>
       <c r="R51" s="6"/>
       <c r="S51" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="52" spans="2:19" x14ac:dyDescent="0.35">
@@ -3705,10 +3697,10 @@
         <v>16</v>
       </c>
       <c r="D52" s="7" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="E52" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F52" s="8">
         <v>46185</v>
@@ -3718,24 +3710,26 @@
       </c>
       <c r="H52" s="12"/>
       <c r="I52" s="6" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="J52" s="6"/>
-      <c r="K52" s="6"/>
-      <c r="L52" s="6"/>
-      <c r="M52" s="6"/>
-      <c r="N52" s="6"/>
-      <c r="O52" s="6"/>
-      <c r="P52" s="6"/>
-      <c r="Q52" s="6"/>
-      <c r="R52" s="6"/>
+      <c r="K52" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="L52" s="21"/>
+      <c r="M52" s="21"/>
+      <c r="N52" s="21"/>
+      <c r="O52" s="21"/>
+      <c r="P52" s="21"/>
+      <c r="Q52" s="21"/>
+      <c r="R52" s="21"/>
       <c r="S52" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="53" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B53" s="6" t="s">
-        <v>20</v>
+        <v>97</v>
       </c>
       <c r="C53" s="6" t="s">
         <v>16</v>
@@ -3744,7 +3738,7 @@
         <v>21</v>
       </c>
       <c r="E53" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F53" s="8">
         <v>46185</v>
@@ -3754,11 +3748,11 @@
       </c>
       <c r="H53" s="12"/>
       <c r="I53" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="J53" s="6"/>
       <c r="K53" s="6" t="s">
-        <v>30</v>
+        <v>106</v>
       </c>
       <c r="L53" s="21"/>
       <c r="M53" s="21"/>
@@ -3768,36 +3762,30 @@
       <c r="Q53" s="21"/>
       <c r="R53" s="21"/>
       <c r="S53" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="54" spans="2:19" x14ac:dyDescent="0.35">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="54" spans="2:19" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B54" s="6" t="s">
-        <v>99</v>
+        <v>20</v>
       </c>
       <c r="C54" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D54" s="7" t="s">
-        <v>21</v>
-      </c>
+      <c r="D54" s="7"/>
       <c r="E54" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F54" s="8">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="G54" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H54" s="12"/>
-      <c r="I54" s="6" t="s">
-        <v>107</v>
-      </c>
+      <c r="I54" s="6"/>
       <c r="J54" s="6"/>
-      <c r="K54" s="6" t="s">
-        <v>108</v>
-      </c>
+      <c r="K54" s="6"/>
       <c r="L54" s="21"/>
       <c r="M54" s="21"/>
       <c r="N54" s="21"/>
@@ -3809,25 +3797,27 @@
         <v>126</v>
       </c>
     </row>
-    <row r="55" spans="2:19" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B55" s="6" t="s">
         <v>20</v>
       </c>
       <c r="C55" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D55" s="7"/>
+      <c r="D55" s="7" t="s">
+        <v>32</v>
+      </c>
       <c r="E55" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F55" s="8">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="G55" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H55" s="12"/>
-      <c r="I55" s="6"/>
+      <c r="H55" s="13"/>
+      <c r="I55" s="50"/>
       <c r="J55" s="6"/>
       <c r="K55" s="6"/>
       <c r="L55" s="21"/>
@@ -3838,30 +3828,30 @@
       <c r="Q55" s="21"/>
       <c r="R55" s="21"/>
       <c r="S55" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="56" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B56" s="6" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C56" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D56" s="7" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="E56" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="F56" s="8">
+        <v>65</v>
+      </c>
+      <c r="F56" s="11">
         <v>46189</v>
       </c>
       <c r="G56" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H56" s="13"/>
-      <c r="I56" s="50"/>
+      <c r="H56" s="12"/>
+      <c r="I56" s="6"/>
       <c r="J56" s="6"/>
       <c r="K56" s="6"/>
       <c r="L56" s="21"/>
@@ -3877,18 +3867,18 @@
     </row>
     <row r="57" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B57" s="6" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C57" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D57" s="7" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="E57" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="F57" s="11">
+        <v>65</v>
+      </c>
+      <c r="F57" s="8">
         <v>46189</v>
       </c>
       <c r="G57" s="7" t="s">
@@ -3911,16 +3901,16 @@
     </row>
     <row r="58" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B58" s="6" t="s">
-        <v>20</v>
+        <v>97</v>
       </c>
       <c r="C58" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D58" s="7" t="s">
-        <v>21</v>
+      <c r="D58" s="34" t="s">
+        <v>214</v>
       </c>
       <c r="E58" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F58" s="8">
         <v>46189</v>
@@ -3929,9 +3919,15 @@
         <v>14</v>
       </c>
       <c r="H58" s="12"/>
-      <c r="I58" s="6"/>
-      <c r="J58" s="6"/>
-      <c r="K58" s="6"/>
+      <c r="I58" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="J58" s="34" t="s">
+        <v>214</v>
+      </c>
+      <c r="K58" s="34" t="s">
+        <v>213</v>
+      </c>
       <c r="L58" s="21"/>
       <c r="M58" s="21"/>
       <c r="N58" s="21"/>
@@ -3940,37 +3936,33 @@
       <c r="Q58" s="21"/>
       <c r="R58" s="21"/>
       <c r="S58" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="59" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B59" s="6" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C59" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D59" s="34" t="s">
-        <v>216</v>
-      </c>
+      <c r="D59" s="7"/>
       <c r="E59" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F59" s="8">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="G59" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H59" s="12"/>
-      <c r="I59" s="15" t="s">
+      <c r="I59" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="J59" s="6"/>
+      <c r="K59" s="6" t="s">
         <v>115</v>
-      </c>
-      <c r="J59" s="34" t="s">
-        <v>216</v>
-      </c>
-      <c r="K59" s="34" t="s">
-        <v>215</v>
       </c>
       <c r="L59" s="21"/>
       <c r="M59" s="21"/>
@@ -3985,27 +3977,29 @@
     </row>
     <row r="60" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B60" s="6" t="s">
-        <v>99</v>
+        <v>57</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D60" s="7"/>
+        <v>11</v>
+      </c>
+      <c r="D60" s="7" t="s">
+        <v>71</v>
+      </c>
       <c r="E60" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F60" s="8">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="G60" s="7" t="s">
-        <v>14</v>
+        <v>66</v>
       </c>
       <c r="H60" s="12"/>
-      <c r="I60" s="6" t="s">
-        <v>104</v>
+      <c r="I60" s="21" t="s">
+        <v>113</v>
       </c>
       <c r="J60" s="6"/>
-      <c r="K60" s="6" t="s">
+      <c r="K60" s="35" t="s">
         <v>117</v>
       </c>
       <c r="L60" s="21"/>
@@ -4021,30 +4015,28 @@
     </row>
     <row r="61" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B61" s="6" t="s">
-        <v>58</v>
+        <v>97</v>
       </c>
       <c r="C61" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D61" s="7" t="s">
-        <v>73</v>
-      </c>
+      <c r="D61" s="7"/>
       <c r="E61" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F61" s="8">
         <v>46191</v>
       </c>
       <c r="G61" s="7" t="s">
-        <v>68</v>
+        <v>14</v>
       </c>
       <c r="H61" s="12"/>
-      <c r="I61" s="21" t="s">
-        <v>115</v>
+      <c r="I61" s="6" t="s">
+        <v>119</v>
       </c>
       <c r="J61" s="6"/>
-      <c r="K61" s="35" t="s">
-        <v>119</v>
+      <c r="K61" s="6" t="s">
+        <v>120</v>
       </c>
       <c r="L61" s="21"/>
       <c r="M61" s="21"/>
@@ -4054,34 +4046,34 @@
       <c r="Q61" s="21"/>
       <c r="R61" s="21"/>
       <c r="S61" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="62" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B62" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C62" s="6" t="s">
+      <c r="B62" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C62" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="D62" s="7"/>
-      <c r="E62" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="F62" s="8">
+      <c r="D62" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="E62" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="F62" s="19">
         <v>46191</v>
       </c>
-      <c r="G62" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="H62" s="12"/>
-      <c r="I62" s="6" t="s">
-        <v>121</v>
+      <c r="G62" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H62" s="20"/>
+      <c r="I62" s="16" t="s">
+        <v>122</v>
       </c>
       <c r="J62" s="6"/>
-      <c r="K62" s="6" t="s">
-        <v>122</v>
-      </c>
+      <c r="K62" s="6"/>
       <c r="L62" s="21"/>
       <c r="M62" s="21"/>
       <c r="N62" s="21"/>
@@ -4090,32 +4082,28 @@
       <c r="Q62" s="21"/>
       <c r="R62" s="21"/>
       <c r="S62" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="63" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B63" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="C63" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="D63" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="E63" s="18" t="s">
-        <v>67</v>
-      </c>
-      <c r="F63" s="19">
+      <c r="B63" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D63" s="7"/>
+      <c r="E63" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="F63" s="8">
         <v>46191</v>
       </c>
-      <c r="G63" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="H63" s="20"/>
-      <c r="I63" s="16" t="s">
-        <v>124</v>
-      </c>
+      <c r="G63" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H63" s="12"/>
+      <c r="I63" s="6"/>
       <c r="J63" s="6"/>
       <c r="K63" s="6"/>
       <c r="L63" s="21"/>
@@ -4126,19 +4114,19 @@
       <c r="Q63" s="21"/>
       <c r="R63" s="21"/>
       <c r="S63" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="64" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B64" s="6" t="s">
-        <v>10</v>
+        <v>97</v>
       </c>
       <c r="C64" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D64" s="7"/>
       <c r="E64" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F64" s="8">
         <v>46191</v>
@@ -4146,10 +4134,12 @@
       <c r="G64" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H64" s="12"/>
+      <c r="H64" s="13"/>
       <c r="I64" s="6"/>
       <c r="J64" s="6"/>
-      <c r="K64" s="6"/>
+      <c r="K64" s="6" t="s">
+        <v>125</v>
+      </c>
       <c r="L64" s="21"/>
       <c r="M64" s="21"/>
       <c r="N64" s="21"/>
@@ -4158,31 +4148,33 @@
       <c r="Q64" s="21"/>
       <c r="R64" s="21"/>
       <c r="S64" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="65" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B65" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C65" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D65" s="7"/>
-      <c r="E65" s="7" t="s">
-        <v>67</v>
+      <c r="B65" s="48" t="s">
+        <v>20</v>
+      </c>
+      <c r="C65" s="48" t="s">
+        <v>11</v>
+      </c>
+      <c r="D65" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E65" s="9" t="s">
+        <v>65</v>
       </c>
       <c r="F65" s="8">
         <v>46191</v>
       </c>
-      <c r="G65" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="H65" s="13"/>
+      <c r="G65" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H65" s="12"/>
       <c r="I65" s="6"/>
       <c r="J65" s="6"/>
       <c r="K65" s="6" t="s">
-        <v>127</v>
+        <v>30</v>
       </c>
       <c r="L65" s="21"/>
       <c r="M65" s="21"/>
@@ -4192,33 +4184,33 @@
       <c r="Q65" s="21"/>
       <c r="R65" s="21"/>
       <c r="S65" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="66" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B66" s="48" t="s">
-        <v>20</v>
-      </c>
-      <c r="C66" s="48" t="s">
-        <v>11</v>
-      </c>
-      <c r="D66" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E66" s="9" t="s">
-        <v>67</v>
+      <c r="B66" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D66" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E66" s="7" t="s">
+        <v>65</v>
       </c>
       <c r="F66" s="8">
-        <v>46191</v>
-      </c>
-      <c r="G66" s="9" t="s">
+        <v>46194</v>
+      </c>
+      <c r="G66" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H66" s="12"/>
       <c r="I66" s="6"/>
       <c r="J66" s="6"/>
       <c r="K66" s="6" t="s">
-        <v>30</v>
+        <v>128</v>
       </c>
       <c r="L66" s="21"/>
       <c r="M66" s="21"/>
@@ -4228,24 +4220,24 @@
       <c r="Q66" s="21"/>
       <c r="R66" s="21"/>
       <c r="S66" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="67" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B67" s="6" t="s">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="C67" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D67" s="7" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E67" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F67" s="8">
-        <v>46194</v>
+        <v>46195</v>
       </c>
       <c r="G67" s="7" t="s">
         <v>14</v>
@@ -4254,7 +4246,7 @@
       <c r="I67" s="6"/>
       <c r="J67" s="6"/>
       <c r="K67" s="6" t="s">
-        <v>130</v>
+        <v>49</v>
       </c>
       <c r="L67" s="21"/>
       <c r="M67" s="21"/>
@@ -4264,24 +4256,24 @@
       <c r="Q67" s="21"/>
       <c r="R67" s="21"/>
       <c r="S67" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="68" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B68" s="6" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C68" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D68" s="7" t="s">
-        <v>12</v>
+        <v>130</v>
       </c>
       <c r="E68" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="F68" s="8">
-        <v>46195</v>
+        <v>65</v>
+      </c>
+      <c r="F68" s="11">
+        <v>46196</v>
       </c>
       <c r="G68" s="7" t="s">
         <v>14</v>
@@ -4289,9 +4281,7 @@
       <c r="H68" s="12"/>
       <c r="I68" s="6"/>
       <c r="J68" s="6"/>
-      <c r="K68" s="6" t="s">
-        <v>50</v>
-      </c>
+      <c r="K68" s="6"/>
       <c r="L68" s="21"/>
       <c r="M68" s="21"/>
       <c r="N68" s="21"/>
@@ -4300,32 +4290,38 @@
       <c r="Q68" s="21"/>
       <c r="R68" s="21"/>
       <c r="S68" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="69" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B69" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C69" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D69" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="E69" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="F69" s="11">
+      <c r="B69" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="C69" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="D69" s="44" t="s">
+        <v>215</v>
+      </c>
+      <c r="E69" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="F69" s="25">
         <v>46196</v>
       </c>
-      <c r="G69" s="7" t="s">
+      <c r="G69" s="24" t="s">
         <v>14</v>
       </c>
       <c r="H69" s="12"/>
-      <c r="I69" s="6"/>
-      <c r="J69" s="6"/>
-      <c r="K69" s="6"/>
+      <c r="I69" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="J69" s="44" t="s">
+        <v>216</v>
+      </c>
+      <c r="K69" s="44" t="s">
+        <v>212</v>
+      </c>
       <c r="L69" s="21"/>
       <c r="M69" s="21"/>
       <c r="N69" s="21"/>
@@ -4334,38 +4330,34 @@
       <c r="Q69" s="21"/>
       <c r="R69" s="21"/>
       <c r="S69" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="70" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B70" s="21" t="s">
-        <v>99</v>
-      </c>
-      <c r="C70" s="21" t="s">
-        <v>11</v>
-      </c>
-      <c r="D70" s="44" t="s">
-        <v>217</v>
-      </c>
-      <c r="E70" s="24" t="s">
-        <v>67</v>
-      </c>
-      <c r="F70" s="25">
+      <c r="B70" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D70" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E70" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="F70" s="8">
         <v>46196</v>
       </c>
-      <c r="G70" s="24" t="s">
+      <c r="G70" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H70" s="12"/>
-      <c r="I70" s="21" t="s">
-        <v>70</v>
-      </c>
-      <c r="J70" s="44" t="s">
-        <v>218</v>
-      </c>
-      <c r="K70" s="44" t="s">
-        <v>214</v>
-      </c>
+      <c r="I70" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="J70" s="6"/>
+      <c r="K70" s="6"/>
       <c r="L70" s="21"/>
       <c r="M70" s="21"/>
       <c r="N70" s="21"/>
@@ -4379,16 +4371,16 @@
     </row>
     <row r="71" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B71" s="6" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C71" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D71" s="7" t="s">
-        <v>73</v>
+        <v>21</v>
       </c>
       <c r="E71" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F71" s="8">
         <v>46196</v>
@@ -4397,11 +4389,11 @@
         <v>14</v>
       </c>
       <c r="H71" s="12"/>
-      <c r="I71" s="6" t="s">
+      <c r="I71" s="50"/>
+      <c r="J71" s="6"/>
+      <c r="K71" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="J71" s="6"/>
-      <c r="K71" s="6"/>
       <c r="L71" s="21"/>
       <c r="M71" s="21"/>
       <c r="N71" s="21"/>
@@ -4410,7 +4402,7 @@
       <c r="Q71" s="21"/>
       <c r="R71" s="21"/>
       <c r="S71" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="72" spans="2:19" x14ac:dyDescent="0.35">
@@ -4418,26 +4410,26 @@
         <v>20</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D72" s="7" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="E72" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F72" s="8">
-        <v>46196</v>
+        <v>46198</v>
       </c>
       <c r="G72" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H72" s="12"/>
-      <c r="I72" s="50"/>
+      <c r="H72" s="13"/>
+      <c r="I72" s="6" t="s">
+        <v>68</v>
+      </c>
       <c r="J72" s="6"/>
-      <c r="K72" s="6" t="s">
-        <v>137</v>
-      </c>
+      <c r="K72" s="6"/>
       <c r="L72" s="21"/>
       <c r="M72" s="21"/>
       <c r="N72" s="21"/>
@@ -4446,7 +4438,7 @@
       <c r="Q72" s="21"/>
       <c r="R72" s="21"/>
       <c r="S72" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="73" spans="2:19" x14ac:dyDescent="0.35">
@@ -4454,24 +4446,24 @@
         <v>20</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D73" s="7" t="s">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="E73" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F73" s="8">
         <v>46198</v>
       </c>
       <c r="G73" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="H73" s="13"/>
-      <c r="I73" s="6" t="s">
-        <v>70</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="H73" s="12">
+        <v>46253</v>
+      </c>
+      <c r="I73" s="6"/>
       <c r="J73" s="6"/>
       <c r="K73" s="6"/>
       <c r="L73" s="21"/>
@@ -4486,30 +4478,30 @@
       </c>
     </row>
     <row r="74" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B74" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C74" s="6" t="s">
+      <c r="B74" s="47" t="s">
+        <v>10</v>
+      </c>
+      <c r="C74" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="D74" s="7" t="s">
-        <v>12</v>
-      </c>
+      <c r="D74" s="7"/>
       <c r="E74" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="F74" s="8">
+        <v>65</v>
+      </c>
+      <c r="F74" s="19">
         <v>46198</v>
       </c>
       <c r="G74" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="H74" s="12">
-        <v>46253</v>
-      </c>
-      <c r="I74" s="6"/>
+        <v>14</v>
+      </c>
+      <c r="H74" s="22"/>
+      <c r="I74" s="6" t="s">
+        <v>59</v>
+      </c>
       <c r="J74" s="6"/>
-      <c r="K74" s="6"/>
+      <c r="K74" s="6" t="s">
+        <v>49</v>
+      </c>
       <c r="L74" s="21"/>
       <c r="M74" s="21"/>
       <c r="N74" s="21"/>
@@ -4518,34 +4510,32 @@
       <c r="Q74" s="21"/>
       <c r="R74" s="21"/>
       <c r="S74" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="75" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B75" s="47" t="s">
+      <c r="B75" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C75" s="47" t="s">
-        <v>16</v>
-      </c>
-      <c r="D75" s="7"/>
+      <c r="C75" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D75" s="7" t="s">
+        <v>21</v>
+      </c>
       <c r="E75" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="F75" s="19">
+        <v>65</v>
+      </c>
+      <c r="F75" s="8">
         <v>46198</v>
       </c>
       <c r="G75" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H75" s="22"/>
-      <c r="I75" s="6" t="s">
-        <v>61</v>
-      </c>
+      <c r="H75" s="12"/>
+      <c r="I75" s="6"/>
       <c r="J75" s="6"/>
-      <c r="K75" s="6" t="s">
-        <v>50</v>
-      </c>
+      <c r="K75" s="6"/>
       <c r="L75" s="21"/>
       <c r="M75" s="21"/>
       <c r="N75" s="21"/>
@@ -4554,7 +4544,7 @@
       <c r="Q75" s="21"/>
       <c r="R75" s="21"/>
       <c r="S75" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="76" spans="2:19" x14ac:dyDescent="0.35">
@@ -4565,21 +4555,27 @@
         <v>11</v>
       </c>
       <c r="D76" s="7" t="s">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="E76" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F76" s="8">
-        <v>46198</v>
+        <v>46202</v>
       </c>
       <c r="G76" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="H76" s="12"/>
-      <c r="I76" s="6"/>
+        <v>66</v>
+      </c>
+      <c r="H76" s="12">
+        <v>46252</v>
+      </c>
+      <c r="I76" s="6" t="s">
+        <v>141</v>
+      </c>
       <c r="J76" s="6"/>
-      <c r="K76" s="6"/>
+      <c r="K76" s="6" t="s">
+        <v>142</v>
+      </c>
       <c r="L76" s="21"/>
       <c r="M76" s="21"/>
       <c r="N76" s="21"/>
@@ -4588,38 +4584,32 @@
       <c r="Q76" s="21"/>
       <c r="R76" s="21"/>
       <c r="S76" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="77" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B77" s="6" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D77" s="7" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E77" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F77" s="8">
         <v>46202</v>
       </c>
       <c r="G77" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="H77" s="12">
-        <v>46252</v>
-      </c>
-      <c r="I77" s="6" t="s">
-        <v>143</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="H77" s="12"/>
+      <c r="I77" s="6"/>
       <c r="J77" s="6"/>
-      <c r="K77" s="6" t="s">
-        <v>144</v>
-      </c>
+      <c r="K77" s="6"/>
       <c r="L77" s="21"/>
       <c r="M77" s="21"/>
       <c r="N77" s="21"/>
@@ -4628,7 +4618,7 @@
       <c r="Q77" s="21"/>
       <c r="R77" s="21"/>
       <c r="S77" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="78" spans="2:19" x14ac:dyDescent="0.35">
@@ -4639,19 +4629,21 @@
         <v>16</v>
       </c>
       <c r="D78" s="7" t="s">
-        <v>73</v>
+        <v>21</v>
       </c>
       <c r="E78" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="F78" s="8">
-        <v>46202</v>
-      </c>
-      <c r="G78" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="F78" s="11">
+        <v>46203</v>
+      </c>
+      <c r="G78" s="23" t="s">
         <v>14</v>
       </c>
       <c r="H78" s="12"/>
-      <c r="I78" s="6"/>
+      <c r="I78" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="J78" s="6"/>
       <c r="K78" s="6"/>
       <c r="L78" s="21"/>
@@ -4667,26 +4659,26 @@
     </row>
     <row r="79" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B79" s="6" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C79" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D79" s="7" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E79" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="F79" s="11">
+        <v>65</v>
+      </c>
+      <c r="F79" s="8">
         <v>46203</v>
       </c>
-      <c r="G79" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="H79" s="12"/>
+      <c r="G79" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H79" s="13"/>
       <c r="I79" s="6" t="s">
-        <v>39</v>
+        <v>105</v>
       </c>
       <c r="J79" s="6"/>
       <c r="K79" s="6"/>
@@ -4698,7 +4690,7 @@
       <c r="Q79" s="21"/>
       <c r="R79" s="21"/>
       <c r="S79" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="80" spans="2:19" x14ac:dyDescent="0.35">
@@ -4708,11 +4700,9 @@
       <c r="C80" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D80" s="7" t="s">
-        <v>12</v>
-      </c>
+      <c r="D80" s="7"/>
       <c r="E80" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F80" s="8">
         <v>46203</v>
@@ -4720,9 +4710,9 @@
       <c r="G80" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H80" s="13"/>
+      <c r="H80" s="12"/>
       <c r="I80" s="6" t="s">
-        <v>107</v>
+        <v>68</v>
       </c>
       <c r="J80" s="6"/>
       <c r="K80" s="6"/>
@@ -4734,29 +4724,31 @@
       <c r="Q80" s="21"/>
       <c r="R80" s="21"/>
       <c r="S80" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="81" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B81" s="6" t="s">
-        <v>10</v>
+        <v>61</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D81" s="7"/>
+        <v>11</v>
+      </c>
+      <c r="D81" s="7" t="s">
+        <v>71</v>
+      </c>
       <c r="E81" s="7" t="s">
-        <v>67</v>
+        <v>148</v>
       </c>
       <c r="F81" s="8">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="G81" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H81" s="12"/>
+      <c r="H81" s="13"/>
       <c r="I81" s="6" t="s">
-        <v>70</v>
+        <v>29</v>
       </c>
       <c r="J81" s="6"/>
       <c r="K81" s="6"/>
@@ -4768,21 +4760,19 @@
       <c r="Q81" s="21"/>
       <c r="R81" s="21"/>
       <c r="S81" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="82" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B82" s="6" t="s">
-        <v>63</v>
+        <v>10</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D82" s="7" t="s">
-        <v>73</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="D82" s="7"/>
       <c r="E82" s="7" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F82" s="8">
         <v>46204</v>
@@ -4790,10 +4780,8 @@
       <c r="G82" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H82" s="13"/>
-      <c r="I82" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="H82" s="12"/>
+      <c r="I82" s="6"/>
       <c r="J82" s="6"/>
       <c r="K82" s="6"/>
       <c r="L82" s="21"/>
@@ -4808,26 +4796,33 @@
       </c>
     </row>
     <row r="83" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="B83" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C83" s="6" t="s">
+      <c r="A83" s="45" t="s">
+        <v>250</v>
+      </c>
+      <c r="B83" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="C83" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="D83" s="7"/>
-      <c r="E83" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="F83" s="8">
+      <c r="D83" s="34" t="s">
+        <v>252</v>
+      </c>
+      <c r="E83" s="24" t="s">
+        <v>148</v>
+      </c>
+      <c r="F83" s="25">
         <v>46204</v>
       </c>
-      <c r="G83" s="7" t="s">
+      <c r="G83" s="24" t="s">
         <v>14</v>
       </c>
       <c r="H83" s="12"/>
-      <c r="I83" s="6"/>
-      <c r="J83" s="6"/>
-      <c r="K83" s="6"/>
+      <c r="I83" s="44"/>
+      <c r="J83" s="51" t="s">
+        <v>251</v>
+      </c>
+      <c r="K83" s="21"/>
       <c r="L83" s="21"/>
       <c r="M83" s="21"/>
       <c r="N83" s="21"/>
@@ -4840,32 +4835,27 @@
       </c>
     </row>
     <row r="84" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A84" s="45" t="s">
-        <v>252</v>
-      </c>
       <c r="B84" s="21" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C84" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="D84" s="34" t="s">
-        <v>254</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="D84" s="24"/>
       <c r="E84" s="24" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F84" s="25">
-        <v>46204</v>
+        <v>46205</v>
       </c>
       <c r="G84" s="24" t="s">
         <v>14</v>
       </c>
       <c r="H84" s="12"/>
-      <c r="I84" s="44"/>
-      <c r="J84" s="51" t="s">
-        <v>253</v>
-      </c>
+      <c r="I84" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="J84" s="21"/>
       <c r="K84" s="21"/>
       <c r="L84" s="21"/>
       <c r="M84" s="21"/>
@@ -4879,28 +4869,32 @@
       </c>
     </row>
     <row r="85" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="B85" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="C85" s="21" t="s">
-        <v>11</v>
-      </c>
-      <c r="D85" s="24"/>
-      <c r="E85" s="24" t="s">
-        <v>150</v>
-      </c>
-      <c r="F85" s="25">
-        <v>46205</v>
-      </c>
-      <c r="G85" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="H85" s="12"/>
-      <c r="I85" s="21" t="s">
-        <v>74</v>
-      </c>
-      <c r="J85" s="21"/>
-      <c r="K85" s="21"/>
+      <c r="B85" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="C85" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="D85" s="26" t="s">
+        <v>12</v>
+      </c>
+      <c r="E85" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="F85" s="27">
+        <v>46210</v>
+      </c>
+      <c r="G85" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="H85" s="49"/>
+      <c r="I85" s="16" t="s">
+        <v>152</v>
+      </c>
+      <c r="J85" s="6"/>
+      <c r="K85" s="36" t="s">
+        <v>117</v>
+      </c>
       <c r="L85" s="21"/>
       <c r="M85" s="21"/>
       <c r="N85" s="21"/>
@@ -4913,32 +4907,28 @@
       </c>
     </row>
     <row r="86" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="B86" s="16" t="s">
+      <c r="B86" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="C86" s="16" t="s">
+      <c r="C86" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="D86" s="26" t="s">
+      <c r="D86" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="E86" s="26" t="s">
-        <v>150</v>
-      </c>
-      <c r="F86" s="27">
-        <v>46210</v>
-      </c>
-      <c r="G86" s="26" t="s">
-        <v>68</v>
-      </c>
-      <c r="H86" s="49"/>
-      <c r="I86" s="16" t="s">
-        <v>154</v>
-      </c>
-      <c r="J86" s="6"/>
-      <c r="K86" s="36" t="s">
-        <v>119</v>
-      </c>
+      <c r="E86" s="24" t="s">
+        <v>148</v>
+      </c>
+      <c r="F86" s="25">
+        <v>46211</v>
+      </c>
+      <c r="G86" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="H86" s="12"/>
+      <c r="I86" s="21"/>
+      <c r="J86" s="21"/>
+      <c r="K86" s="21"/>
       <c r="L86" s="21"/>
       <c r="M86" s="21"/>
       <c r="N86" s="21"/>
@@ -4947,24 +4937,24 @@
       <c r="Q86" s="21"/>
       <c r="R86" s="21"/>
       <c r="S86" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="87" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B87" s="21" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C87" s="21" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D87" s="24" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="E87" s="24" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F87" s="25">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="G87" s="24" t="s">
         <v>14</v>
@@ -4986,16 +4976,16 @@
     </row>
     <row r="88" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B88" s="21" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C88" s="21" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D88" s="24" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E88" s="24" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F88" s="25">
         <v>46212</v>
@@ -5020,26 +5010,32 @@
     </row>
     <row r="89" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B89" s="21" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C89" s="21" t="s">
         <v>16</v>
       </c>
       <c r="D89" s="24" t="s">
-        <v>12</v>
+        <v>130</v>
       </c>
       <c r="E89" s="24" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F89" s="25">
         <v>46212</v>
       </c>
       <c r="G89" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="H89" s="12"/>
-      <c r="I89" s="21"/>
-      <c r="J89" s="21"/>
+        <v>66</v>
+      </c>
+      <c r="H89" s="22">
+        <v>46259</v>
+      </c>
+      <c r="I89" s="21" t="s">
+        <v>157</v>
+      </c>
+      <c r="J89" s="21" t="s">
+        <v>158</v>
+      </c>
       <c r="K89" s="21"/>
       <c r="L89" s="21"/>
       <c r="M89" s="21"/>
@@ -5054,33 +5050,35 @@
     </row>
     <row r="90" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B90" s="21" t="s">
-        <v>20</v>
+        <v>57</v>
       </c>
       <c r="C90" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="D90" s="24" t="s">
-        <v>132</v>
+      <c r="D90" s="44" t="s">
+        <v>249</v>
       </c>
       <c r="E90" s="24" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F90" s="25">
         <v>46212</v>
       </c>
       <c r="G90" s="24" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="H90" s="22">
-        <v>46259</v>
+        <v>46258</v>
       </c>
       <c r="I90" s="21" t="s">
-        <v>159</v>
-      </c>
-      <c r="J90" s="21" t="s">
         <v>160</v>
       </c>
-      <c r="K90" s="21"/>
+      <c r="J90" s="44" t="s">
+        <v>249</v>
+      </c>
+      <c r="K90" s="44" t="s">
+        <v>248</v>
+      </c>
       <c r="L90" s="21"/>
       <c r="M90" s="21"/>
       <c r="N90" s="21"/>
@@ -5089,39 +5087,37 @@
       <c r="Q90" s="21"/>
       <c r="R90" s="21"/>
       <c r="S90" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="91" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B91" s="21" t="s">
-        <v>58</v>
+        <v>10</v>
       </c>
       <c r="C91" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="D91" s="44" t="s">
-        <v>251</v>
+        <v>11</v>
+      </c>
+      <c r="D91" s="24" t="s">
+        <v>12</v>
       </c>
       <c r="E91" s="24" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F91" s="25">
         <v>46212</v>
       </c>
       <c r="G91" s="24" t="s">
-        <v>68</v>
-      </c>
-      <c r="H91" s="22">
-        <v>46258</v>
+        <v>87</v>
+      </c>
+      <c r="H91" s="12">
+        <v>46259</v>
       </c>
       <c r="I91" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="J91" s="44" t="s">
-        <v>251</v>
-      </c>
-      <c r="K91" s="44" t="s">
-        <v>250</v>
+      <c r="J91" s="21"/>
+      <c r="K91" s="53" t="s">
+        <v>163</v>
       </c>
       <c r="L91" s="21"/>
       <c r="M91" s="21"/>
@@ -5131,38 +5127,33 @@
       <c r="Q91" s="21"/>
       <c r="R91" s="21"/>
       <c r="S91" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="92" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A92" s="45" t="s">
+        <v>253</v>
+      </c>
       <c r="B92" s="21" t="s">
         <v>10</v>
       </c>
       <c r="C92" s="21" t="s">
-        <v>11</v>
-      </c>
-      <c r="D92" s="24" t="s">
-        <v>12</v>
-      </c>
+        <v>205</v>
+      </c>
+      <c r="D92" s="44"/>
       <c r="E92" s="24" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F92" s="25">
         <v>46212</v>
       </c>
       <c r="G92" s="24" t="s">
-        <v>89</v>
-      </c>
-      <c r="H92" s="12">
-        <v>46259</v>
-      </c>
-      <c r="I92" s="21" t="s">
-        <v>164</v>
-      </c>
-      <c r="J92" s="21"/>
-      <c r="K92" s="53" t="s">
-        <v>165</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="H92" s="12"/>
+      <c r="I92" s="44"/>
+      <c r="J92" s="44"/>
+      <c r="K92" s="21"/>
       <c r="L92" s="21"/>
       <c r="M92" s="21"/>
       <c r="N92" s="21"/>
@@ -5175,28 +5166,25 @@
       </c>
     </row>
     <row r="93" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A93" s="45" t="s">
-        <v>255</v>
-      </c>
       <c r="B93" s="21" t="s">
         <v>10</v>
       </c>
       <c r="C93" s="21" t="s">
-        <v>207</v>
-      </c>
-      <c r="D93" s="44"/>
+        <v>11</v>
+      </c>
+      <c r="D93" s="24"/>
       <c r="E93" s="24" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F93" s="25">
-        <v>46212</v>
+        <v>46216</v>
       </c>
       <c r="G93" s="24" t="s">
         <v>14</v>
       </c>
       <c r="H93" s="12"/>
-      <c r="I93" s="44"/>
-      <c r="J93" s="44"/>
+      <c r="I93" s="21"/>
+      <c r="J93" s="21"/>
       <c r="K93" s="21"/>
       <c r="L93" s="21"/>
       <c r="M93" s="21"/>
@@ -5211,14 +5199,16 @@
     </row>
     <row r="94" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B94" s="21" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C94" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="D94" s="24"/>
+      <c r="D94" s="24" t="s">
+        <v>71</v>
+      </c>
       <c r="E94" s="24" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F94" s="25">
         <v>46216</v>
@@ -5226,8 +5216,10 @@
       <c r="G94" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="H94" s="12"/>
-      <c r="I94" s="21"/>
+      <c r="H94" s="13"/>
+      <c r="I94" s="21" t="s">
+        <v>133</v>
+      </c>
       <c r="J94" s="21"/>
       <c r="K94" s="21"/>
       <c r="L94" s="21"/>
@@ -5238,33 +5230,35 @@
       <c r="Q94" s="21"/>
       <c r="R94" s="21"/>
       <c r="S94" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="95" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B95" s="21" t="s">
-        <v>20</v>
+        <v>57</v>
       </c>
       <c r="C95" s="21" t="s">
         <v>11</v>
       </c>
       <c r="D95" s="24" t="s">
-        <v>73</v>
+        <v>12</v>
       </c>
       <c r="E95" s="24" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F95" s="25">
-        <v>46216</v>
+        <v>46219</v>
       </c>
       <c r="G95" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="H95" s="13"/>
+      <c r="H95" s="12"/>
       <c r="I95" s="21" t="s">
-        <v>135</v>
-      </c>
-      <c r="J95" s="21"/>
+        <v>167</v>
+      </c>
+      <c r="J95" s="44" t="s">
+        <v>218</v>
+      </c>
       <c r="K95" s="21"/>
       <c r="L95" s="21"/>
       <c r="M95" s="21"/>
@@ -5279,31 +5273,35 @@
     </row>
     <row r="96" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B96" s="21" t="s">
-        <v>58</v>
+        <v>10</v>
       </c>
       <c r="C96" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="D96" s="24" t="s">
-        <v>12</v>
+      <c r="D96" s="44" t="s">
+        <v>218</v>
       </c>
       <c r="E96" s="24" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F96" s="25">
         <v>46219</v>
       </c>
       <c r="G96" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="H96" s="12"/>
+        <v>87</v>
+      </c>
+      <c r="H96" s="22">
+        <v>46265</v>
+      </c>
       <c r="I96" s="21" t="s">
+        <v>162</v>
+      </c>
+      <c r="J96" s="44" t="s">
+        <v>217</v>
+      </c>
+      <c r="K96" s="21" t="s">
         <v>169</v>
       </c>
-      <c r="J96" s="44" t="s">
-        <v>220</v>
-      </c>
-      <c r="K96" s="21"/>
       <c r="L96" s="21"/>
       <c r="M96" s="21"/>
       <c r="N96" s="21"/>
@@ -5312,40 +5310,36 @@
       <c r="Q96" s="21"/>
       <c r="R96" s="21"/>
       <c r="S96" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="97" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B97" s="21" t="s">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="C97" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="D97" s="44" t="s">
-        <v>220</v>
+      <c r="D97" s="24" t="s">
+        <v>171</v>
       </c>
       <c r="E97" s="24" t="s">
-        <v>150</v>
-      </c>
-      <c r="F97" s="25">
-        <v>46219</v>
+        <v>148</v>
+      </c>
+      <c r="F97" s="28">
+        <v>46223</v>
       </c>
       <c r="G97" s="24" t="s">
-        <v>89</v>
-      </c>
-      <c r="H97" s="22">
-        <v>46265</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="H97" s="12"/>
       <c r="I97" s="21" t="s">
-        <v>164</v>
-      </c>
-      <c r="J97" s="44" t="s">
-        <v>219</v>
-      </c>
-      <c r="K97" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="J97" s="21" t="s">
         <v>171</v>
       </c>
+      <c r="K97" s="21"/>
       <c r="L97" s="21"/>
       <c r="M97" s="21"/>
       <c r="N97" s="21"/>
@@ -5354,23 +5348,23 @@
       <c r="Q97" s="21"/>
       <c r="R97" s="21"/>
       <c r="S97" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="98" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B98" s="21" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="C98" s="21" t="s">
         <v>11</v>
       </c>
       <c r="D98" s="24" t="s">
-        <v>173</v>
+        <v>21</v>
       </c>
       <c r="E98" s="24" t="s">
-        <v>150</v>
-      </c>
-      <c r="F98" s="28">
+        <v>148</v>
+      </c>
+      <c r="F98" s="25">
         <v>46223</v>
       </c>
       <c r="G98" s="24" t="s">
@@ -5378,11 +5372,9 @@
       </c>
       <c r="H98" s="12"/>
       <c r="I98" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="J98" s="21" t="s">
         <v>173</v>
       </c>
+      <c r="J98" s="21"/>
       <c r="K98" s="21"/>
       <c r="L98" s="21"/>
       <c r="M98" s="21"/>
@@ -5392,34 +5384,36 @@
       <c r="Q98" s="21"/>
       <c r="R98" s="21"/>
       <c r="S98" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="99" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="B99" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="C99" s="21" t="s">
+      <c r="B99" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C99" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D99" s="24" t="s">
-        <v>21</v>
-      </c>
-      <c r="E99" s="24" t="s">
-        <v>150</v>
-      </c>
-      <c r="F99" s="25">
-        <v>46223</v>
-      </c>
-      <c r="G99" s="24" t="s">
+      <c r="D99" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E99" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="F99" s="8">
+        <v>46224</v>
+      </c>
+      <c r="G99" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H99" s="12"/>
-      <c r="I99" s="21" t="s">
+      <c r="I99" s="6"/>
+      <c r="J99" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="J99" s="21"/>
-      <c r="K99" s="21"/>
+      <c r="K99" s="6" t="s">
+        <v>176</v>
+      </c>
       <c r="L99" s="21"/>
       <c r="M99" s="21"/>
       <c r="N99" s="21"/>
@@ -5428,35 +5422,40 @@
       <c r="Q99" s="21"/>
       <c r="R99" s="21"/>
       <c r="S99" t="s">
-        <v>209</v>
+        <v>260</v>
       </c>
     </row>
     <row r="100" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A100" s="41" t="s">
+        <v>254</v>
+      </c>
       <c r="B100" s="6" t="s">
-        <v>99</v>
+        <v>20</v>
       </c>
       <c r="C100" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D100" s="7" t="s">
-        <v>32</v>
+        <v>16</v>
+      </c>
+      <c r="D100" s="34" t="s">
+        <v>255</v>
       </c>
       <c r="E100" s="7" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F100" s="8">
         <v>46224</v>
       </c>
-      <c r="G100" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="H100" s="12"/>
-      <c r="I100" s="6"/>
-      <c r="J100" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="K100" s="6" t="s">
-        <v>178</v>
+      <c r="G100" s="42" t="s">
+        <v>87</v>
+      </c>
+      <c r="H100" s="12">
+        <v>46274</v>
+      </c>
+      <c r="I100" s="34"/>
+      <c r="J100" s="34" t="s">
+        <v>255</v>
+      </c>
+      <c r="K100" s="34" t="s">
+        <v>256</v>
       </c>
       <c r="L100" s="21"/>
       <c r="M100" s="21"/>
@@ -5466,104 +5465,97 @@
       <c r="Q100" s="21"/>
       <c r="R100" s="21"/>
       <c r="S100" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="101" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A101" s="41" t="s">
-        <v>256</v>
-      </c>
       <c r="B101" s="6" t="s">
         <v>20</v>
       </c>
       <c r="C101" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D101" s="34" t="s">
-        <v>257</v>
+        <v>11</v>
+      </c>
+      <c r="D101" s="7" t="s">
+        <v>178</v>
       </c>
       <c r="E101" s="7" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F101" s="8">
-        <v>46224</v>
-      </c>
-      <c r="G101" s="42" t="s">
-        <v>89</v>
+        <v>46227</v>
+      </c>
+      <c r="G101" s="7" t="s">
+        <v>66</v>
       </c>
       <c r="H101" s="12">
-        <v>46274</v>
-      </c>
-      <c r="I101" s="34"/>
-      <c r="J101" s="34" t="s">
-        <v>257</v>
-      </c>
-      <c r="K101" s="34" t="s">
-        <v>258</v>
-      </c>
-      <c r="L101" s="21"/>
-      <c r="M101" s="21"/>
-      <c r="N101" s="21"/>
-      <c r="O101" s="21"/>
-      <c r="P101" s="21"/>
-      <c r="Q101" s="21"/>
-      <c r="R101" s="21"/>
+        <v>46255</v>
+      </c>
+      <c r="I101" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="J101" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="K101" s="6"/>
+      <c r="L101" s="6"/>
+      <c r="M101" s="6"/>
+      <c r="N101" s="6"/>
+      <c r="O101" s="6"/>
+      <c r="P101" s="6"/>
+      <c r="Q101" s="6"/>
+      <c r="R101" s="6"/>
       <c r="S101" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="102" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B102" s="6" t="s">
-        <v>20</v>
+        <v>97</v>
       </c>
       <c r="C102" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D102" s="7" t="s">
-        <v>180</v>
+        <v>21</v>
       </c>
       <c r="E102" s="7" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F102" s="8">
         <v>46227</v>
       </c>
       <c r="G102" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="H102" s="12">
-        <v>46255</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="H102" s="12"/>
       <c r="I102" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="J102" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="J102" s="6"/>
+      <c r="K102" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="K102" s="6"/>
-      <c r="L102" s="6"/>
-      <c r="M102" s="6"/>
-      <c r="N102" s="6"/>
-      <c r="O102" s="6"/>
-      <c r="P102" s="6"/>
-      <c r="Q102" s="6"/>
-      <c r="R102" s="6"/>
+      <c r="L102" s="21"/>
+      <c r="M102" s="21"/>
+      <c r="N102" s="21"/>
+      <c r="O102" s="21"/>
+      <c r="P102" s="21"/>
+      <c r="Q102" s="21"/>
+      <c r="R102" s="21"/>
       <c r="S102" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="103" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B103" s="6" t="s">
-        <v>99</v>
+        <v>57</v>
       </c>
       <c r="C103" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D103" s="7" t="s">
-        <v>21</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="D103" s="7"/>
       <c r="E103" s="7" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F103" s="8">
         <v>46227</v>
@@ -5572,9 +5564,7 @@
         <v>14</v>
       </c>
       <c r="H103" s="12"/>
-      <c r="I103" s="6" t="s">
-        <v>49</v>
-      </c>
+      <c r="I103" s="6"/>
       <c r="J103" s="6"/>
       <c r="K103" s="6" t="s">
         <v>182</v>
@@ -5587,19 +5577,21 @@
       <c r="Q103" s="21"/>
       <c r="R103" s="21"/>
       <c r="S103" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="104" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B104" s="6" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="C104" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D104" s="7"/>
+      <c r="D104" s="7" t="s">
+        <v>12</v>
+      </c>
       <c r="E104" s="7" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F104" s="8">
         <v>46227</v>
@@ -5608,10 +5600,12 @@
         <v>14</v>
       </c>
       <c r="H104" s="12"/>
-      <c r="I104" s="6"/>
+      <c r="I104" s="6" t="s">
+        <v>184</v>
+      </c>
       <c r="J104" s="6"/>
       <c r="K104" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="L104" s="21"/>
       <c r="M104" s="21"/>
@@ -5621,35 +5615,37 @@
       <c r="Q104" s="21"/>
       <c r="R104" s="21"/>
       <c r="S104" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="105" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B105" s="6" t="s">
-        <v>20</v>
+        <v>97</v>
       </c>
       <c r="C105" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D105" s="7" t="s">
-        <v>12</v>
+        <v>187</v>
       </c>
       <c r="E105" s="7" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F105" s="8">
-        <v>46227</v>
+        <v>46231</v>
       </c>
       <c r="G105" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H105" s="12"/>
       <c r="I105" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="J105" s="6"/>
+        <v>188</v>
+      </c>
+      <c r="J105" s="6" t="s">
+        <v>187</v>
+      </c>
       <c r="K105" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="L105" s="21"/>
       <c r="M105" s="21"/>
@@ -5659,37 +5655,36 @@
       <c r="Q105" s="21"/>
       <c r="R105" s="21"/>
       <c r="S105" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="106" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A106" s="46" t="s">
+        <v>258</v>
+      </c>
       <c r="B106" s="6" t="s">
-        <v>99</v>
+        <v>20</v>
       </c>
       <c r="C106" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D106" s="7" t="s">
-        <v>189</v>
+        <v>11</v>
+      </c>
+      <c r="D106" s="34" t="s">
+        <v>257</v>
       </c>
       <c r="E106" s="7" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F106" s="8">
-        <v>46231</v>
-      </c>
-      <c r="G106" s="7" t="s">
+        <v>46232</v>
+      </c>
+      <c r="G106" s="42" t="s">
         <v>14</v>
       </c>
       <c r="H106" s="12"/>
-      <c r="I106" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="J106" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="K106" s="6" t="s">
-        <v>191</v>
+      <c r="I106" s="34"/>
+      <c r="J106" s="34"/>
+      <c r="K106" s="35" t="s">
+        <v>259</v>
       </c>
       <c r="L106" s="21"/>
       <c r="M106" s="21"/>
@@ -5699,37 +5694,36 @@
       <c r="Q106" s="21"/>
       <c r="R106" s="21"/>
       <c r="S106" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="107" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A107" s="46" t="s">
-        <v>260</v>
-      </c>
       <c r="B107" s="6" t="s">
-        <v>20</v>
+        <v>97</v>
       </c>
       <c r="C107" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D107" s="34" t="s">
-        <v>259</v>
+      <c r="D107" s="7" t="s">
+        <v>191</v>
       </c>
       <c r="E107" s="7" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F107" s="8">
-        <v>46232</v>
-      </c>
-      <c r="G107" s="42" t="s">
+        <v>46233</v>
+      </c>
+      <c r="G107" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H107" s="12"/>
-      <c r="I107" s="34"/>
-      <c r="J107" s="34"/>
-      <c r="K107" s="35" t="s">
-        <v>261</v>
-      </c>
+      <c r="I107" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="J107" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="K107" s="6"/>
       <c r="L107" s="21"/>
       <c r="M107" s="21"/>
       <c r="N107" s="21"/>
@@ -5738,32 +5732,30 @@
       <c r="Q107" s="21"/>
       <c r="R107" s="21"/>
       <c r="S107" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="108" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B108" s="6" t="s">
-        <v>99</v>
+        <v>20</v>
       </c>
       <c r="C108" s="6" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D108" s="7" t="s">
         <v>193</v>
       </c>
       <c r="E108" s="7" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F108" s="8">
         <v>46233</v>
       </c>
       <c r="G108" s="7" t="s">
-        <v>14</v>
+        <v>66</v>
       </c>
       <c r="H108" s="12"/>
-      <c r="I108" s="6" t="s">
-        <v>124</v>
-      </c>
+      <c r="I108" s="6"/>
       <c r="J108" s="6" t="s">
         <v>193</v>
       </c>
@@ -5776,12 +5768,12 @@
       <c r="Q108" s="21"/>
       <c r="R108" s="21"/>
       <c r="S108" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="109" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B109" s="6" t="s">
-        <v>20</v>
+        <v>97</v>
       </c>
       <c r="C109" s="6" t="s">
         <v>16</v>
@@ -5790,20 +5782,22 @@
         <v>195</v>
       </c>
       <c r="E109" s="7" t="s">
-        <v>150</v>
+        <v>196</v>
       </c>
       <c r="F109" s="8">
-        <v>46233</v>
+        <v>46244</v>
       </c>
       <c r="G109" s="7" t="s">
-        <v>68</v>
+        <v>14</v>
       </c>
       <c r="H109" s="12"/>
       <c r="I109" s="6"/>
       <c r="J109" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="K109" s="6"/>
+        <v>197</v>
+      </c>
+      <c r="K109" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="L109" s="21"/>
       <c r="M109" s="21"/>
       <c r="N109" s="21"/>
@@ -5812,36 +5806,32 @@
       <c r="Q109" s="21"/>
       <c r="R109" s="21"/>
       <c r="S109" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="110" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B110" s="6" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C110" s="6" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D110" s="7" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="E110" s="7" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="F110" s="8">
-        <v>46244</v>
+        <v>46247</v>
       </c>
       <c r="G110" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H110" s="12"/>
       <c r="I110" s="6"/>
-      <c r="J110" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="K110" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="J110" s="6"/>
+      <c r="K110" s="6"/>
       <c r="L110" s="21"/>
       <c r="M110" s="21"/>
       <c r="N110" s="21"/>
@@ -5850,21 +5840,19 @@
       <c r="Q110" s="21"/>
       <c r="R110" s="21"/>
       <c r="S110" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="111" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B111" s="6" t="s">
-        <v>99</v>
+        <v>20</v>
       </c>
       <c r="C111" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D111" s="7" t="s">
-        <v>201</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="D111" s="7"/>
       <c r="E111" s="7" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="F111" s="8">
         <v>46247</v>
@@ -5884,29 +5872,35 @@
       <c r="Q111" s="21"/>
       <c r="R111" s="21"/>
       <c r="S111" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="112" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B112" s="6" t="s">
-        <v>20</v>
+        <v>97</v>
       </c>
       <c r="C112" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D112" s="7"/>
+        <v>11</v>
+      </c>
+      <c r="D112" s="7" t="s">
+        <v>202</v>
+      </c>
       <c r="E112" s="7" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="F112" s="8">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="G112" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H112" s="12"/>
-      <c r="I112" s="6"/>
-      <c r="J112" s="6"/>
+      <c r="I112" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="J112" s="6" t="s">
+        <v>202</v>
+      </c>
       <c r="K112" s="6"/>
       <c r="L112" s="21"/>
       <c r="M112" s="21"/>
@@ -5916,34 +5910,34 @@
       <c r="Q112" s="21"/>
       <c r="R112" s="21"/>
       <c r="S112" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="113" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B113" s="6" t="s">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="C113" s="6" t="s">
-        <v>11</v>
+        <v>205</v>
       </c>
       <c r="D113" s="7" t="s">
-        <v>204</v>
+        <v>12</v>
       </c>
       <c r="E113" s="7" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="F113" s="8">
-        <v>46248</v>
+        <v>46251</v>
       </c>
       <c r="G113" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H113" s="12"/>
       <c r="I113" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="J113" s="6" t="s">
-        <v>204</v>
+        <v>18</v>
+      </c>
+      <c r="J113" s="52" t="s">
+        <v>206</v>
       </c>
       <c r="K113" s="6"/>
       <c r="L113" s="21"/>
@@ -5954,46 +5948,27 @@
       <c r="Q113" s="21"/>
       <c r="R113" s="21"/>
       <c r="S113" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="114" spans="2:19" x14ac:dyDescent="0.35">
-      <c r="B114" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C114" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="D114" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="E114" s="7" t="s">
-        <v>198</v>
-      </c>
-      <c r="F114" s="8">
-        <v>46251</v>
-      </c>
-      <c r="G114" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="H114" s="12"/>
-      <c r="I114" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="J114" s="52" t="s">
-        <v>208</v>
-      </c>
-      <c r="K114" s="6"/>
-      <c r="L114" s="21"/>
-      <c r="M114" s="21"/>
-      <c r="N114" s="21"/>
-      <c r="O114" s="21"/>
-      <c r="P114" s="21"/>
-      <c r="Q114" s="21"/>
-      <c r="R114" s="21"/>
-      <c r="S114" t="s">
-        <v>276</v>
-      </c>
+      <c r="B114" s="29"/>
+      <c r="C114" s="29"/>
+      <c r="D114" s="30"/>
+      <c r="E114" s="30"/>
+      <c r="F114" s="31"/>
+      <c r="G114" s="30"/>
+      <c r="H114" s="32"/>
+      <c r="I114" s="29"/>
+      <c r="J114" s="29"/>
+      <c r="K114" s="29"/>
+      <c r="L114" s="29"/>
+      <c r="M114" s="29"/>
+      <c r="N114" s="29"/>
+      <c r="O114" s="29"/>
+      <c r="P114" s="29"/>
+      <c r="Q114" s="29"/>
+      <c r="R114" s="29"/>
     </row>
     <row r="115" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B115" s="29"/>
@@ -7477,56 +7452,37 @@
       <c r="Q192" s="29"/>
       <c r="R192" s="29"/>
     </row>
-    <row r="193" spans="2:18" x14ac:dyDescent="0.35">
-      <c r="B193" s="29"/>
-      <c r="C193" s="29"/>
-      <c r="D193" s="30"/>
-      <c r="E193" s="30"/>
-      <c r="F193" s="31"/>
-      <c r="G193" s="30"/>
-      <c r="H193" s="32"/>
-      <c r="I193" s="29"/>
-      <c r="J193" s="29"/>
-      <c r="K193" s="29"/>
-      <c r="L193" s="29"/>
-      <c r="M193" s="29"/>
-      <c r="N193" s="29"/>
-      <c r="O193" s="29"/>
-      <c r="P193" s="29"/>
-      <c r="Q193" s="29"/>
-      <c r="R193" s="29"/>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L198">
-    <sortCondition ref="F2:F198"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L197">
+    <sortCondition ref="F2:F197"/>
   </sortState>
   <phoneticPr fontId="13" type="noConversion"/>
   <dataValidations count="10">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D85:D99 D115:D1048576 D50:D58 D80:D83 D102 D109 D60:D78 D30:D37 D39:D48 D4:D6 D8:D28" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D84:D98 D114:D1048576 D49:D57 D79:D82 D101 D108 D59:D77 D29:D36 D38:D47 D4:D6 D8:D27" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"ECE,ChemE,Phy,EE,CS,BME,BA,Others,"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E105:E1048576 E4:E103" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E104:E1048576 E4:E102" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"6月,5月,7月,8月,4月,"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="B65:B114 B2:B63" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" sqref="B64:B113 B2:B62" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"北京,上海,广州,武汉,沈阳"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="B64" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" sqref="B63" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"北京,上海,广州,武汉,沈阳"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B115:B193" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B114:B192" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"北京,上海,广州,武汉,沈阳"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="C65:C114 C2:C63" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" sqref="C64:C113 C2:C62" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"PhD,Master,Bachelor"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="C64" xr:uid="{00000000-0002-0000-0000-000008000000}">
+    <dataValidation type="list" sqref="C63" xr:uid="{00000000-0002-0000-0000-000008000000}">
       <formula1>"PhD,Master,Bachelor"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C115:C193" xr:uid="{00000000-0002-0000-0000-000009000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C114:C192" xr:uid="{00000000-0002-0000-0000-000009000000}">
       <formula1>"PhD,Master,Bachelor"</formula1>
     </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F1048576 H4:H1048576" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H4:H1048576 F4:F1048576" xr:uid="{00000000-0002-0000-0000-000000000000}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G4:G1048576" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Check,Approve,Issue,"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
feat: release Checkee Hall data 20260916-v001
</commit_message>
<xml_diff>
--- a/data/checkmate/hall_fame.xlsx
+++ b/data/checkmate/hall_fame.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\projects_2027\checkee_2026\data\checkmate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F58A4127-BC96-40B9-AAE6-DB08711EB5C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E305144-FDF2-4E24-9D9D-14365C0A63AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6980" yWindow="5440" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="836" uniqueCount="284">
   <si>
     <t>地点</t>
   </si>
@@ -1161,6 +1161,70 @@
   </si>
   <si>
     <t>金牌狗啃包</t>
+    <phoneticPr fontId="13" type="noConversion"/>
+  </si>
+  <si>
+    <t>椰</t>
+    <phoneticPr fontId="13" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>9.1updated</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>接使馆电话更新</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>i20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>，9.11</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>ap</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>，9.14</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>is</t>
+    </r>
     <phoneticPr fontId="13" type="noConversion"/>
   </si>
 </sst>
@@ -3272,6 +3336,9 @@
       </c>
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A41" s="45" t="s">
+        <v>282</v>
+      </c>
       <c r="B41" s="6" t="s">
         <v>20</v>
       </c>
@@ -3290,14 +3357,18 @@
       <c r="G41" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="H41" s="13"/>
+      <c r="H41" s="13">
+        <v>46279</v>
+      </c>
       <c r="I41" s="6" t="s">
         <v>51</v>
       </c>
       <c r="J41" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="K41" s="6"/>
+      <c r="K41" s="34" t="s">
+        <v>283</v>
+      </c>
       <c r="L41" s="6"/>
       <c r="M41" s="6"/>
       <c r="N41" s="6"/>

</xml_diff>